<commit_message>
Add client photos to five butterfly valve galleries and HP v03 literature
From the client's "Pictures to be added to website" package:
- Chem-Tek, Hi-Tek, HP, Performance and 52DF galleries keep their
  current main image and add the new photos in place of duplicate views
- HP Series literature updated to 501-24 v03

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAX-SEAL-main/catalog/MAXSEAL_CATALOG.xlsx
+++ b/MAX-SEAL-main/catalog/MAXSEAL_CATALOG.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2861" uniqueCount="1201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2877" uniqueCount="1228">
   <si>
     <t>Id</t>
   </si>
@@ -2844,10 +2844,13 @@
     <t>hp-series</t>
   </si>
   <si>
-    <t>High Performance Series Catalog (501-24 High Performance Series_v02 COMPRESSED.pdf)</t>
-  </si>
-  <si>
-    <t>/assets/maxseal/docs/501-24 High Performance Series_v02 COMPRESSED.pdf</t>
+    <t>High Performance Series Catalog (501-24 High Performance Series_v03.pdf)</t>
+  </si>
+  <si>
+    <t>4.0 MB</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/docs/501-24 High Performance Series_v03.pdf</t>
   </si>
   <si>
     <t>d16</t>
@@ -3516,6 +3519,18 @@
     <t>View 3</t>
   </si>
   <si>
+    <t>/assets/maxseal/products/Series 52DF Large Angle.png</t>
+  </si>
+  <si>
+    <t>Large – Angle</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Series 52DF Large Front.png</t>
+  </si>
+  <si>
+    <t>Large – Front</t>
+  </si>
+  <si>
     <t>/assets/maxseal/products/Hayward BYV Series Butterfly Valve Angle.png</t>
   </si>
   <si>
@@ -3556,6 +3571,72 @@
   </si>
   <si>
     <t>/assets/maxseal/products/Chem-Flo Series Ball Valve.png</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Performance Series Handle.png</t>
+  </si>
+  <si>
+    <t>With Handle</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Performance Series Cutaway.png</t>
+  </si>
+  <si>
+    <t>Cutaway</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Performance Series 6in Bare.png</t>
+  </si>
+  <si>
+    <t>6" Bare</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Chem-Tek Series Bare.png</t>
+  </si>
+  <si>
+    <t>Bare Valve</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Chem-Tek Series Actuated.png</t>
+  </si>
+  <si>
+    <t>Actuated</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Chem-Tek Series Top Works.png</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/HP Series Double Offset Actuated.jpg</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/HP Series Lug Scotch Yoke.jpg</t>
+  </si>
+  <si>
+    <t>Scotch Yoke</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/HP Series Actuated Lineup.png</t>
+  </si>
+  <si>
+    <t>Lineup</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Hi-Tek Series Actuated.png</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Hi-Tek Series Stainless Gear Operated.png</t>
+  </si>
+  <si>
+    <t>Stainless</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Hi-Tek Series Scotch Yoke.png</t>
+  </si>
+  <si>
+    <t>/assets/maxseal/products/Hi-Tek Series AirCon Actuated.png</t>
+  </si>
+  <si>
+    <t>AirCon Actuated</t>
   </si>
   <si>
     <t>Section</t>
@@ -4636,10 +4717,12 @@
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
+      <c r="H16" s="1" t="s">
+        <v>936</v>
+      </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1" t="s">
-        <v>936</v>
+        <v>937</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" t="s">
@@ -4648,16 +4731,16 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>937</v>
+        <v>938</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>938</v>
+        <v>939</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>939</v>
+        <v>940</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>281</v>
@@ -4667,7 +4750,7 @@
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1" t="s">
-        <v>940</v>
+        <v>941</v>
       </c>
       <c r="K17" s="1"/>
       <c r="L17" t="s">
@@ -4676,16 +4759,16 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>941</v>
+        <v>942</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>942</v>
+        <v>943</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>943</v>
+        <v>944</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>289</v>
@@ -4695,7 +4778,7 @@
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="K18" s="1"/>
       <c r="L18" t="s">
@@ -4704,16 +4787,16 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>946</v>
+        <v>947</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>947</v>
+        <v>948</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>299</v>
@@ -4723,7 +4806,7 @@
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
       <c r="J19" s="1" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="K19" s="1"/>
       <c r="L19" t="s">
@@ -4732,16 +4815,16 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>950</v>
+        <v>951</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>310</v>
@@ -4751,7 +4834,7 @@
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
       <c r="J20" s="1" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" t="s">
@@ -4760,16 +4843,16 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>954</v>
+        <v>955</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>955</v>
+        <v>956</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>319</v>
@@ -4779,7 +4862,7 @@
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
       <c r="J21" s="1" t="s">
-        <v>956</v>
+        <v>957</v>
       </c>
       <c r="K21" s="1"/>
       <c r="L21" t="s">
@@ -4788,16 +4871,16 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>957</v>
+        <v>958</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>958</v>
+        <v>959</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>959</v>
+        <v>960</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>250</v>
@@ -4807,7 +4890,7 @@
       <c r="H22" s="1"/>
       <c r="I22" s="1"/>
       <c r="J22" s="1" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
       <c r="K22" s="1"/>
       <c r="L22" t="s">
@@ -4816,16 +4899,16 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>206</v>
@@ -4837,7 +4920,7 @@
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
       <c r="J23" s="1" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="K23" s="1"/>
       <c r="L23" t="s">
@@ -4846,16 +4929,16 @@
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>206</v>
@@ -4863,11 +4946,11 @@
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="I24" s="1"/>
       <c r="J24" s="1" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="K24" s="1"/>
       <c r="L24" t="s">
@@ -4876,28 +4959,28 @@
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>354</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
       <c r="J25" s="1" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="K25" s="1"/>
       <c r="L25" t="s">
@@ -4906,28 +4989,28 @@
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>361</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
       <c r="K26" s="1"/>
       <c r="L26" t="s">
@@ -4936,28 +5019,28 @@
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>425</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="G27" s="1"/>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="K27" s="1"/>
       <c r="L27" t="s">
@@ -4966,30 +5049,30 @@
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>902</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="1" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="I28" s="1"/>
       <c r="J28" s="1" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
       <c r="K28" s="1"/>
       <c r="L28" t="s">
@@ -4998,16 +5081,16 @@
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>230</v>
@@ -5019,13 +5102,13 @@
         <v>104</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="I29" s="1" t="s">
         <v>104</v>
       </c>
       <c r="J29" s="1" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="K29" s="1" t="s">
         <v>104</v>
@@ -5039,16 +5122,16 @@
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>902</v>
@@ -5060,13 +5143,13 @@
         <v>104</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="I30" s="1" t="s">
         <v>104</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
       <c r="K30" s="1" t="s">
         <v>104</v>
@@ -5080,16 +5163,16 @@
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>895</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>1004</v>
+        <v>1005</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>230</v>
@@ -5101,13 +5184,13 @@
         <v>104</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>104</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="K31" s="1" t="s">
         <v>104</v>
@@ -5121,16 +5204,16 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>853</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>195</v>
@@ -5148,7 +5231,7 @@
         <v>104</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>104</v>
@@ -5162,16 +5245,16 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>895</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>902</v>
@@ -5183,13 +5266,13 @@
         <v>104</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>104</v>
       </c>
       <c r="J33" s="1" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="K33" s="1" t="s">
         <v>104</v>
@@ -5203,16 +5286,16 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>882</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>902</v>
@@ -5224,13 +5307,13 @@
         <v>104</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="I34" s="1" t="s">
         <v>104</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
       <c r="K34" s="1" t="s">
         <v>104</v>
@@ -5244,16 +5327,16 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>902</v>
@@ -5271,7 +5354,7 @@
         <v>104</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="K35" s="1" t="s">
         <v>104</v>
@@ -5356,16 +5439,16 @@
         <v>445</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>846</v>
@@ -5386,60 +5469,60 @@
     </row>
     <row r="3" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>902</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
       <c r="I3" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>902</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="I4" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
     </row>
   </sheetData>
@@ -5478,63 +5561,63 @@
         <v>447</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>847</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="K1" s="4" t="s">
         <v>845</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>853</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="H2" s="6" t="s">
         <v>32</v>
@@ -5542,22 +5625,22 @@
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
       <c r="K3" s="6" t="s">
         <v>864</v>
@@ -5565,25 +5648,25 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="L4" s="6" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
       <c r="N4" s="6" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
     </row>
   </sheetData>
@@ -5610,7 +5693,7 @@
         <v>445</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>6</v>
@@ -6530,45 +6613,45 @@
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>35</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>128</v>
@@ -6576,22 +6659,22 @@
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>41</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="G3" s="6" t="s">
         <v>144</v>
@@ -6599,22 +6682,22 @@
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>157</v>
@@ -6622,22 +6705,22 @@
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>167</v>
@@ -6645,22 +6728,22 @@
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>180</v>
@@ -6668,22 +6751,22 @@
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="G7" s="6" t="s">
         <v>195</v>
@@ -6691,22 +6774,22 @@
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>206</v>
@@ -6714,22 +6797,22 @@
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>653</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G9" s="6" t="s">
         <v>651</v>
@@ -6737,22 +6820,22 @@
     </row>
     <row r="10" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>657</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G10" s="6" t="s">
         <v>655</v>
@@ -6760,22 +6843,22 @@
     </row>
     <row r="11" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>661</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G11" s="6" t="s">
         <v>659</v>
@@ -6783,22 +6866,22 @@
     </row>
     <row r="12" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>665</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G12" s="6" t="s">
         <v>663</v>
@@ -6806,22 +6889,22 @@
     </row>
     <row r="13" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="D13" s="6" t="s">
         <v>669</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G13" s="6" t="s">
         <v>667</v>
@@ -6829,22 +6912,22 @@
     </row>
     <row r="14" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>673</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G14" s="6" t="s">
         <v>671</v>
@@ -6852,22 +6935,22 @@
     </row>
     <row r="15" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="D15" s="6" t="s">
         <v>677</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>675</v>
@@ -6875,22 +6958,22 @@
     </row>
     <row r="16" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>681</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G16" s="6" t="s">
         <v>679</v>
@@ -6898,22 +6981,22 @@
     </row>
     <row r="17" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>685</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G17" s="6" t="s">
         <v>683</v>
@@ -6921,22 +7004,22 @@
     </row>
     <row r="18" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>689</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G18" s="6" t="s">
         <v>687</v>
@@ -6944,22 +7027,22 @@
     </row>
     <row r="19" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>693</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G19" s="6" t="s">
         <v>691</v>
@@ -6967,22 +7050,22 @@
     </row>
     <row r="20" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>697</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G20" s="6" t="s">
         <v>695</v>
@@ -6990,22 +7073,22 @@
     </row>
     <row r="21" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>701</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>699</v>
@@ -7013,45 +7096,45 @@
     </row>
     <row r="22" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
     </row>
     <row r="23" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>859</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="G23" s="6" t="s">
         <v>852</v>
@@ -7059,22 +7142,22 @@
     </row>
     <row r="24" ht="18.75" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>860</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="G24" s="6" t="s">
         <v>852</v>
@@ -7091,7 +7174,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:D80"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.453125"/>
   <cols>
     <col min="1" max="1" width="14.01" style="1" customWidth="1"/>
@@ -7122,7 +7205,7 @@
         <v>35</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
@@ -7136,7 +7219,7 @@
         <v>35</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D3" s="1">
         <v>2</v>
@@ -7150,7 +7233,7 @@
         <v>35</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="D4" s="1">
         <v>3</v>
@@ -7164,7 +7247,7 @@
         <v>41</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D5" s="1">
         <v>1</v>
@@ -7178,7 +7261,7 @@
         <v>41</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D6" s="1">
         <v>2</v>
@@ -7192,7 +7275,7 @@
         <v>41</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="D7" s="1">
         <v>3</v>
@@ -7206,7 +7289,7 @@
         <v>46</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D8" s="1">
         <v>1</v>
@@ -7217,10 +7300,10 @@
         <v>157</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>46</v>
+        <v>1160</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>1157</v>
+        <v>1161</v>
       </c>
       <c r="D9" s="1">
         <v>2</v>
@@ -7231,10 +7314,10 @@
         <v>157</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>46</v>
+        <v>1162</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>1158</v>
+        <v>1163</v>
       </c>
       <c r="D10" s="1">
         <v>3</v>
@@ -7248,7 +7331,7 @@
         <v>50</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
@@ -7262,7 +7345,7 @@
         <v>50</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D12" s="1">
         <v>2</v>
@@ -7276,7 +7359,7 @@
         <v>50</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="D13" s="1">
         <v>3</v>
@@ -7290,7 +7373,7 @@
         <v>54</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D14" s="1">
         <v>1</v>
@@ -7301,10 +7384,10 @@
         <v>180</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1159</v>
+        <v>1164</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>1160</v>
+        <v>1165</v>
       </c>
       <c r="D15" s="1">
         <v>2</v>
@@ -7315,10 +7398,10 @@
         <v>180</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>1161</v>
+        <v>1166</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>1162</v>
+        <v>1167</v>
       </c>
       <c r="D16" s="1">
         <v>3</v>
@@ -7332,7 +7415,7 @@
         <v>58</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D17" s="1">
         <v>1</v>
@@ -7343,10 +7426,10 @@
         <v>195</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>1163</v>
+        <v>1168</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>1160</v>
+        <v>1165</v>
       </c>
       <c r="D18" s="1">
         <v>2</v>
@@ -7357,10 +7440,10 @@
         <v>195</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>1164</v>
+        <v>1169</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>1165</v>
+        <v>1170</v>
       </c>
       <c r="D19" s="1">
         <v>3</v>
@@ -7371,10 +7454,10 @@
         <v>195</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>1166</v>
+        <v>1171</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>1167</v>
+        <v>1172</v>
       </c>
       <c r="D20" s="1">
         <v>4</v>
@@ -7388,7 +7471,7 @@
         <v>63</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D21" s="1">
         <v>1</v>
@@ -7399,10 +7482,10 @@
         <v>206</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>1168</v>
+        <v>1173</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>1169</v>
+        <v>1174</v>
       </c>
       <c r="D22" s="1">
         <v>2</v>
@@ -7413,10 +7496,10 @@
         <v>206</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>1170</v>
+        <v>1175</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>1171</v>
+        <v>1176</v>
       </c>
       <c r="D23" s="1">
         <v>3</v>
@@ -7427,7 +7510,7 @@
         <v>206</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>1172</v>
+        <v>1177</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>821</v>
@@ -7444,7 +7527,7 @@
         <v>66</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D25" s="1">
         <v>1</v>
@@ -7458,7 +7541,7 @@
         <v>66</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D26" s="1">
         <v>2</v>
@@ -7472,7 +7555,7 @@
         <v>66</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="D27" s="1">
         <v>3</v>
@@ -7486,7 +7569,7 @@
         <v>237</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D28" s="1">
         <v>1</v>
@@ -7497,10 +7580,10 @@
         <v>230</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>237</v>
+        <v>1178</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>1157</v>
+        <v>1179</v>
       </c>
       <c r="D29" s="1">
         <v>2</v>
@@ -7511,10 +7594,10 @@
         <v>230</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>237</v>
+        <v>1180</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>1158</v>
+        <v>1181</v>
       </c>
       <c r="D30" s="1">
         <v>3</v>
@@ -7522,16 +7605,16 @@
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>247</v>
+        <v>1182</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>1156</v>
+        <v>1183</v>
       </c>
       <c r="D31" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7545,7 +7628,7 @@
         <v>1157</v>
       </c>
       <c r="D32" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7559,21 +7642,21 @@
         <v>1158</v>
       </c>
       <c r="D33" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>1156</v>
+        <v>1159</v>
       </c>
       <c r="D34" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7587,7 +7670,7 @@
         <v>1157</v>
       </c>
       <c r="D35" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7601,21 +7684,21 @@
         <v>1158</v>
       </c>
       <c r="D36" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>1156</v>
+        <v>1159</v>
       </c>
       <c r="D37" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7629,7 +7712,7 @@
         <v>1157</v>
       </c>
       <c r="D38" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7637,41 +7720,41 @@
         <v>258</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>265</v>
+        <v>1184</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>1158</v>
+        <v>1185</v>
       </c>
       <c r="D39" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>278</v>
+        <v>1186</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>1156</v>
+        <v>1187</v>
       </c>
       <c r="D40" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>271</v>
+        <v>258</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>278</v>
+        <v>1188</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>1157</v>
+        <v>1172</v>
       </c>
       <c r="D41" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -7682,63 +7765,63 @@
         <v>278</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D42" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>288</v>
+        <v>1189</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>1156</v>
+        <v>1187</v>
       </c>
       <c r="D43" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>288</v>
+        <v>1190</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>1157</v>
+        <v>1191</v>
       </c>
       <c r="D44" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>288</v>
+        <v>1192</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>1158</v>
+        <v>1193</v>
       </c>
       <c r="D45" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D46" s="1">
         <v>1</v>
@@ -7746,13 +7829,13 @@
     </row>
     <row r="47" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="D47" s="1">
         <v>2</v>
@@ -7760,13 +7843,13 @@
     </row>
     <row r="48" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>296</v>
+        <v>288</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="D48" s="1">
         <v>3</v>
@@ -7774,13 +7857,13 @@
     </row>
     <row r="49" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
       <c r="D49" s="1">
         <v>1</v>
@@ -7788,13 +7871,13 @@
     </row>
     <row r="50" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>306</v>
+        <v>1194</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>1157</v>
+        <v>1187</v>
       </c>
       <c r="D50" s="1">
         <v>2</v>
@@ -7802,13 +7885,13 @@
     </row>
     <row r="51" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>306</v>
+        <v>1195</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>1158</v>
+        <v>1196</v>
       </c>
       <c r="D51" s="1">
         <v>3</v>
@@ -7816,337 +7899,407 @@
     </row>
     <row r="52" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>310</v>
+        <v>289</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>317</v>
+        <v>1197</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>1156</v>
+        <v>1191</v>
       </c>
       <c r="D52" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>310</v>
+        <v>289</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>317</v>
+        <v>1198</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>1157</v>
+        <v>1199</v>
       </c>
       <c r="D53" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D54" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>41</v>
+        <v>306</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D55" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>319</v>
+        <v>299</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>41</v>
+        <v>306</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="D56" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>41</v>
+        <v>317</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D57" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>331</v>
+        <v>310</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>72</v>
+        <v>317</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D58" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>331</v>
+        <v>310</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>72</v>
+        <v>317</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="D59" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D60" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>340</v>
+        <v>319</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D61" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>340</v>
+        <v>319</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="D62" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D63" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>354</v>
+        <v>331</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D64" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>354</v>
+        <v>331</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="D65" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
-        <v>354</v>
+        <v>340</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D66" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>361</v>
+        <v>340</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D67" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>361</v>
+        <v>340</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="D68" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>361</v>
+        <v>354</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D69" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
-        <v>371</v>
+        <v>354</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D70" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>371</v>
+        <v>354</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="D71" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>371</v>
+        <v>361</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="D72" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>379</v>
+        <v>361</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>1156</v>
+        <v>1158</v>
       </c>
       <c r="D73" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
-        <v>379</v>
+        <v>361</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>1157</v>
+        <v>1159</v>
       </c>
       <c r="D74" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D75" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>1158</v>
+      </c>
+      <c r="D76" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="77" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>1159</v>
+      </c>
+      <c r="D77" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="B75" s="1" t="s">
+      <c r="B78" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C75" s="1" t="s">
+      <c r="C78" s="1" t="s">
+        <v>1157</v>
+      </c>
+      <c r="D78" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>1158</v>
       </c>
-      <c r="D75" s="1">
+      <c r="D79" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" ht="15" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>1159</v>
+      </c>
+      <c r="D80" s="1">
         <v>3</v>
       </c>
     </row>
@@ -8170,114 +8323,114 @@
   <sheetData>
     <row r="1" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>1173</v>
+        <v>1200</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1174</v>
+        <v>1201</v>
       </c>
     </row>
     <row r="2" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>1175</v>
+        <v>1202</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>1176</v>
+        <v>1203</v>
       </c>
     </row>
     <row r="3" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>1177</v>
+        <v>1204</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>1178</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="4" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>1179</v>
+        <v>1206</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>1180</v>
+        <v>1207</v>
       </c>
     </row>
     <row r="5" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>1181</v>
+        <v>1208</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>1182</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="6" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>1183</v>
+        <v>1210</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>1184</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="7" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>1185</v>
+        <v>1212</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>1186</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="8" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>1187</v>
+        <v>1214</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>1188</v>
+        <v>1215</v>
       </c>
     </row>
     <row r="9" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>1189</v>
+        <v>1216</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>1190</v>
+        <v>1217</v>
       </c>
     </row>
     <row r="10" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>1191</v>
+        <v>1218</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>1192</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="11" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>1193</v>
+        <v>1220</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>1194</v>
+        <v>1221</v>
       </c>
     </row>
     <row r="12" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
-        <v>1195</v>
+        <v>1222</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>1196</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="13" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>1197</v>
+        <v>1224</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>1198</v>
+        <v>1225</v>
       </c>
     </row>
     <row r="14" ht="18.75" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>1199</v>
+        <v>1226</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>1200</v>
+        <v>1227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Remove Cryogenic series and Stem Extensions from the website
- Set PROD-018 (Cryogenic) and PROD-029 (Stem Extensions) inactive and drop
  related-product links pointing at them
- Hide the cryogenic catalog (d20) and drop PROD-029 from the Easy-Link doc
- Add "Cryogenic Series Valves available upon request." note on High
  Performance, linking to the Support form with Cryogenic preselected
- Remove the Custom Stem Extensions service card from Solutions
- Search skips documents hidden from the Catalog page

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAX-SEAL-main/catalog/MAXSEAL_CATALOG.xlsx
+++ b/MAX-SEAL-main/catalog/MAXSEAL_CATALOG.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3146" uniqueCount="1394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="1394">
   <si>
     <t>Id</t>
   </si>
@@ -3090,7 +3090,7 @@
     <t>Mounting / Manual Override Catalog (150-22 Easy Link for Max-Seal Compressed.pdf)</t>
   </si>
   <si>
-    <t>PROD-026,PROD-027,PROD-028,PROD-029</t>
+    <t>PROD-026,PROD-027,PROD-028</t>
   </si>
   <si>
     <t>/assets/maxseal/docs/150-22 Easy Link for Max-Seal Compressed.pdf</t>
@@ -5364,7 +5364,7 @@
       </c>
       <c r="K21" s="1"/>
       <c r="L21" t="s">
-        <v>675</v>
+        <v>899</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -6334,7 +6334,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.453125"/>
   <cols>
     <col min="1" max="1" width="14.01" style="1" customWidth="1"/>
@@ -6586,13 +6586,13 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>332</v>
-      </c>
       <c r="C23" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -6600,10 +6600,10 @@
         <v>290</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>280</v>
+        <v>302</v>
       </c>
       <c r="C24" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -6611,10 +6611,10 @@
         <v>290</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="C25" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -6622,32 +6622,32 @@
         <v>290</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="C26" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>323</v>
+        <v>280</v>
       </c>
       <c r="C27" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B28" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>332</v>
-      </c>
       <c r="C28" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -6655,10 +6655,10 @@
         <v>302</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>280</v>
+        <v>312</v>
       </c>
       <c r="C29" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -6666,43 +6666,43 @@
         <v>302</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>290</v>
+        <v>323</v>
       </c>
       <c r="C30" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>312</v>
+        <v>280</v>
       </c>
       <c r="C31" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>302</v>
+        <v>312</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>323</v>
+        <v>290</v>
       </c>
       <c r="C32" s="1">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="B33" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>332</v>
-      </c>
       <c r="C33" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -6710,59 +6710,59 @@
         <v>312</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>280</v>
+        <v>323</v>
       </c>
       <c r="C34" s="1">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="C35" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
       <c r="C36" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>312</v>
+        <v>323</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>323</v>
+        <v>302</v>
       </c>
       <c r="C37" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>332</v>
-      </c>
       <c r="C38" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>280</v>
@@ -6773,7 +6773,7 @@
     </row>
     <row r="40" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>290</v>
@@ -6784,7 +6784,7 @@
     </row>
     <row r="41" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>302</v>
@@ -6795,7 +6795,7 @@
     </row>
     <row r="42" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>312</v>
@@ -6806,10 +6806,10 @@
     </row>
     <row r="43" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="B43" s="1" t="s">
         <v>323</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>332</v>
       </c>
       <c r="C43" s="1">
         <v>5</v>
@@ -6817,10 +6817,10 @@
     </row>
     <row r="44" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>332</v>
+        <v>227</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>280</v>
+        <v>215</v>
       </c>
       <c r="C44" s="1">
         <v>1</v>
@@ -6828,10 +6828,10 @@
     </row>
     <row r="45" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>332</v>
+        <v>227</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>290</v>
+        <v>204</v>
       </c>
       <c r="C45" s="1">
         <v>2</v>
@@ -6839,10 +6839,10 @@
     </row>
     <row r="46" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>332</v>
+        <v>227</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>302</v>
+        <v>189</v>
       </c>
       <c r="C46" s="1">
         <v>3</v>
@@ -6850,32 +6850,32 @@
     </row>
     <row r="47" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>332</v>
+        <v>353</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>312</v>
+        <v>394</v>
       </c>
       <c r="C47" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>332</v>
+        <v>353</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>323</v>
+        <v>386</v>
       </c>
       <c r="C48" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>227</v>
+        <v>375</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>215</v>
+        <v>394</v>
       </c>
       <c r="C49" s="1">
         <v>1</v>
@@ -6883,76 +6883,76 @@
     </row>
     <row r="50" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>227</v>
+        <v>375</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>204</v>
+        <v>353</v>
       </c>
       <c r="C50" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>227</v>
+        <v>386</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>189</v>
+        <v>394</v>
       </c>
       <c r="C51" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="B52" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="B52" s="1" t="s">
-        <v>394</v>
-      </c>
       <c r="C52" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B53" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="B53" s="1" t="s">
-        <v>386</v>
-      </c>
       <c r="C53" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="B54" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>394</v>
-      </c>
       <c r="C54" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>375</v>
+        <v>394</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>353</v>
+        <v>386</v>
       </c>
       <c r="C55" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="C56" s="1">
         <v>1</v>
@@ -6960,10 +6960,10 @@
     </row>
     <row r="57" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>386</v>
+        <v>375</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>353</v>
+        <v>414</v>
       </c>
       <c r="C57" s="1">
         <v>2</v>
@@ -6971,276 +6971,177 @@
     </row>
     <row r="58" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>394</v>
+        <v>375</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>353</v>
+        <v>424</v>
       </c>
       <c r="C58" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>375</v>
       </c>
       <c r="C59" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>394</v>
+        <v>404</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>386</v>
+        <v>414</v>
       </c>
       <c r="C60" s="1">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>375</v>
+        <v>404</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>404</v>
+        <v>424</v>
       </c>
       <c r="C61" s="1">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="B62" s="1" t="s">
-        <v>414</v>
-      </c>
       <c r="C62" s="1">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>375</v>
+        <v>414</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>424</v>
+        <v>404</v>
       </c>
       <c r="C63" s="1">
-        <v>3</v>
+        <v>10</v>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
-        <v>375</v>
+        <v>414</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>434</v>
+        <v>424</v>
       </c>
       <c r="C64" s="1">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
-        <v>404</v>
+        <v>424</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>375</v>
       </c>
       <c r="C65" s="1">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>414</v>
-      </c>
       <c r="C66" s="1">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
-        <v>404</v>
+        <v>424</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>424</v>
+        <v>414</v>
       </c>
       <c r="C67" s="1">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
-        <v>404</v>
+        <v>434</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>434</v>
+        <v>375</v>
       </c>
       <c r="C68" s="1">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
-        <v>414</v>
+        <v>434</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>375</v>
+        <v>404</v>
       </c>
       <c r="C69" s="1">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
+        <v>434</v>
+      </c>
+      <c r="B70" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>404</v>
-      </c>
       <c r="C70" s="1">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
-        <v>414</v>
+        <v>434</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>424</v>
       </c>
       <c r="C71" s="1">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
-        <v>414</v>
+        <v>394</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>434</v>
+        <v>463</v>
       </c>
       <c r="C72" s="1">
-        <v>12</v>
+        <v>90</v>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
-        <v>424</v>
+        <v>463</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>375</v>
+        <v>394</v>
       </c>
       <c r="C73" s="1">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="74" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="C74" s="1">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="75" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="C75" s="1">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="76" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="C76" s="1">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="77" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A77" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>375</v>
-      </c>
-      <c r="C77" s="1">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="78" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A78" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="C78" s="1">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="79" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A79" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="C79" s="1">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="80" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A80" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="B80" s="1" t="s">
-        <v>424</v>
-      </c>
-      <c r="C80" s="1">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="81" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A81" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="B81" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="C81" s="1">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="82" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A82" s="1" t="s">
-        <v>463</v>
-      </c>
-      <c r="B82" s="1" t="s">
-        <v>394</v>
-      </c>
-      <c r="C82" s="1">
         <v>91</v>
       </c>
     </row>
@@ -11758,7 +11659,7 @@
         <v>152</v>
       </c>
       <c r="T19" s="1" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="U19" s="1" t="b">
         <f>FALSE()</f>
@@ -12331,7 +12232,7 @@
         <v>442</v>
       </c>
       <c r="T29" s="1" t="s">
-        <v>12</v>
+        <v>67</v>
       </c>
       <c r="V29" s="2">
         <v>5</v>

</xml_diff>

<commit_message>
Filter Regulators: straighten With Gauge photo, label SMC models
- Rotate the AW40 photo 0.76 deg so cap and drain line up vertically
- Gallery labels: Filter Regulator -> SMC AW20-N02C-2Z-A,
  With Gauge -> SMC AW40-N04C-Z-A (client markup)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/MAX-SEAL-main/catalog/MAXSEAL_CATALOG.xlsx
+++ b/MAX-SEAL-main/catalog/MAXSEAL_CATALOG.xlsx
@@ -4065,13 +4065,13 @@
     <t>/assets/maxseal/products/automation/Filter Regulator.png</t>
   </si>
   <si>
-    <t>Filter Regulator</t>
+    <t>SMC AW20-N02C-2Z-A</t>
   </si>
   <si>
     <t>/assets/maxseal/products/automation/Filter Regulator with Gauge.png</t>
   </si>
   <si>
-    <t>With Gauge</t>
+    <t>SMC AW40-N04C-Z-A</t>
   </si>
   <si>
     <t>/assets/maxseal/products/automation/Couplers Set Screws.png</t>

</xml_diff>